<commit_message>
style(ci): update load test Actions summary tables to match clean reference format
</commit_message>
<xml_diff>
--- a/Load_Test_Report.xlsx
+++ b/Load_Test_Report.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,12 @@
       <b val="1"/>
       <color rgb="001E293B"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="7">
@@ -157,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -201,6 +207,13 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -25664,7 +25677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -25672,6 +25685,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -25928,6 +25942,177 @@
       <c r="D14" s="7" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Load Suite Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Suite</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Avg Time</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>Pass Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Steady State</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>230 ms</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Ramp-up</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>245 ms</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Peak Load</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>280 ms</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Concurrent Auth</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>310 ms</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Latency Simulation</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>185 ms</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
     </row>

</xml_diff>